<commit_message>
Sync Forms export and update outputs
</commit_message>
<xml_diff>
--- a/PeerGrading/Input/form_exports/forms_responses.xlsx
+++ b/PeerGrading/Input/form_exports/forms_responses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uzh-my.sharepoint.com/personal/renjie_cui_business_uzh_ch/Documents/PeerGrading/Input/form_exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="318" documentId="8_{9C3C9BE7-B8B4-430B-A3DC-C1A29F196D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3EAD73C-6D11-41A0-9508-F46B9360AE44}"/>
+  <xr:revisionPtr revIDLastSave="333" documentId="8_{9C3C9BE7-B8B4-430B-A3DC-C1A29F196D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CBD8D65-4695-4C34-92BB-16C2C2188FF8}"/>
   <bookViews>
     <workbookView xWindow="17280" yWindow="-16200" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7518" uniqueCount="1423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7713" uniqueCount="1462">
   <si>
     <t>Responseid</t>
   </si>
@@ -4305,6 +4305,123 @@
   </si>
   <si>
     <t>2026-03-04T19:28:41.7544099Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:32:23.2161673Z</t>
+  </si>
+  <si>
+    <t>The information was well prepared and clearly presented.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:32:23.2162078Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:34:10.7835417Z</t>
+  </si>
+  <si>
+    <t>The speaker showed good confidence while presenting.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:34:10.7835848Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:35:18.4540848Z</t>
+  </si>
+  <si>
+    <t>Good balance between visuals and spoken explanation.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:35:18.4541380Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:36:42.3827453Z</t>
+  </si>
+  <si>
+    <t>The presentation was interesting and engaging.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:36:42.3828101Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:34.3910725Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:34.3911378Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:42.6974093Z</t>
+  </si>
+  <si>
+    <t>The presentation showed good preparation and effort.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:42.6974503Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:38:55.0830185Z</t>
+  </si>
+  <si>
+    <t>The speaker communicated the ideas clearly and effectively.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:38:55.0830703Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:39:43.5485937Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:39:43.5486326Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:40:29.1895567Z</t>
+  </si>
+  <si>
+    <t>The examples helped to understand the topic better.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:40:29.1896101Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:12.7058905Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:12.7059302Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:43.6373925Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:43.6374339Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:49.2567103Z</t>
+  </si>
+  <si>
+    <t>Very technical presentation but the key points were explained clearly and effectively.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:49.2567497Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:11.3387463Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:11.3387876Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:40.9457496Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:40.9457885Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:48.3346651Z</t>
+  </si>
+  <si>
+    <t>Well delivered and easy to follow.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:48.3347398Z</t>
   </si>
 </sst>
 </file>
@@ -4408,8 +4525,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="responses" displayName="responses" ref="A1:N617" totalsRowShown="0">
-  <autoFilter ref="A1:N617" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="responses" displayName="responses" ref="A1:N632" totalsRowShown="0">
+  <autoFilter ref="A1:N632" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Responseid" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="SubmittedAt"/>
@@ -4727,7 +4844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N617"/>
+  <dimension ref="A1:N632"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="14" width="20" bestFit="1" customWidth="1"/>
@@ -31706,7 +31823,7 @@
       </c>
     </row>
     <row r="614" spans="1:14">
-      <c r="A614" s="5">
+      <c r="A614">
         <v>618</v>
       </c>
       <c r="B614" s="1" t="s">
@@ -31750,7 +31867,7 @@
       </c>
     </row>
     <row r="615" spans="1:14">
-      <c r="A615" s="5">
+      <c r="A615">
         <v>619</v>
       </c>
       <c r="B615" s="1" t="s">
@@ -31794,7 +31911,7 @@
       </c>
     </row>
     <row r="616" spans="1:14">
-      <c r="A616" s="5">
+      <c r="A616">
         <v>620</v>
       </c>
       <c r="B616" s="1" t="s">
@@ -31838,7 +31955,7 @@
       </c>
     </row>
     <row r="617" spans="1:14">
-      <c r="A617" s="5">
+      <c r="A617">
         <v>621</v>
       </c>
       <c r="B617" s="1" t="s">
@@ -31879,6 +31996,666 @@
       </c>
       <c r="N617" s="4" t="s">
         <v>1422</v>
+      </c>
+    </row>
+    <row r="618" spans="1:14">
+      <c r="A618" s="5">
+        <v>622</v>
+      </c>
+      <c r="B618" s="1" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C618" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D618" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E618" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G618" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H618" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J618" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M618" s="3" t="s">
+        <v>1424</v>
+      </c>
+      <c r="N618" s="4" t="s">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="619" spans="1:14">
+      <c r="A619" s="5">
+        <v>623</v>
+      </c>
+      <c r="B619" s="1" t="s">
+        <v>1426</v>
+      </c>
+      <c r="C619" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D619" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E619" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G619" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H619" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K619" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M619" s="3" t="s">
+        <v>1427</v>
+      </c>
+      <c r="N619" s="4" t="s">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="620" spans="1:14">
+      <c r="A620" s="5">
+        <v>624</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C620" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D620" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E620" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J620" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K620" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M620" s="3" t="s">
+        <v>1430</v>
+      </c>
+      <c r="N620" s="4" t="s">
+        <v>1431</v>
+      </c>
+    </row>
+    <row r="621" spans="1:14">
+      <c r="A621" s="5">
+        <v>625</v>
+      </c>
+      <c r="B621" s="1" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C621" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D621" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E621" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="F621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G621" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J621" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K621" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M621" s="3" t="s">
+        <v>1433</v>
+      </c>
+      <c r="N621" s="4" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="622" spans="1:14">
+      <c r="A622" s="5">
+        <v>626</v>
+      </c>
+      <c r="B622" s="1" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C622" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D622" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E622" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M622" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N622" s="4" t="s">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="623" spans="1:14">
+      <c r="A623" s="5">
+        <v>627</v>
+      </c>
+      <c r="B623" s="1" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C623" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D623" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E623" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="F623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J623" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M623" s="3" t="s">
+        <v>1438</v>
+      </c>
+      <c r="N623" s="4" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="624" spans="1:14">
+      <c r="A624" s="5">
+        <v>628</v>
+      </c>
+      <c r="B624" s="1" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C624" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D624" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E624" s="2" t="s">
+        <v>945</v>
+      </c>
+      <c r="F624" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M624" s="3" t="s">
+        <v>1441</v>
+      </c>
+      <c r="N624" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="625" spans="1:14">
+      <c r="A625" s="5">
+        <v>629</v>
+      </c>
+      <c r="B625" s="1" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C625" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D625" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E625" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M625" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N625" s="4" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="626" spans="1:14">
+      <c r="A626" s="5">
+        <v>630</v>
+      </c>
+      <c r="B626" s="1" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C626" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D626" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E626" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G626" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K626" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M626" s="3" t="s">
+        <v>1446</v>
+      </c>
+      <c r="N626" s="4" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="627" spans="1:14">
+      <c r="A627" s="5">
+        <v>631</v>
+      </c>
+      <c r="B627" s="1" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C627" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D627" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E627" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M627" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N627" s="4" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="628" spans="1:14">
+      <c r="A628" s="5">
+        <v>632</v>
+      </c>
+      <c r="B628" s="1" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C628" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D628" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E628" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="F628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M628" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N628" s="4" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="629" spans="1:14">
+      <c r="A629" s="5">
+        <v>633</v>
+      </c>
+      <c r="B629" s="1" t="s">
+        <v>1452</v>
+      </c>
+      <c r="C629" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D629" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E629" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="F629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H629" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I629" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M629" s="3" t="s">
+        <v>1453</v>
+      </c>
+      <c r="N629" s="4" t="s">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="630" spans="1:14">
+      <c r="A630" s="5">
+        <v>634</v>
+      </c>
+      <c r="B630" s="1" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C630" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D630" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E630" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="F630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M630" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N630" s="4" t="s">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="631" spans="1:14">
+      <c r="A631" s="5">
+        <v>635</v>
+      </c>
+      <c r="B631" s="1" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C631" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D631" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E631" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M631" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N631" s="4" t="s">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="632" spans="1:14">
+      <c r="A632" s="5">
+        <v>636</v>
+      </c>
+      <c r="B632" s="1" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C632" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D632" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E632" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="F632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M632" s="3" t="s">
+        <v>1460</v>
+      </c>
+      <c r="N632" s="4" t="s">
+        <v>1461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync Forms export and update outputs (#8)
Co-authored-by: RenjieCui <71599592+RenjieCui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PeerGrading/Input/form_exports/forms_responses.xlsx
+++ b/PeerGrading/Input/form_exports/forms_responses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uzh-my.sharepoint.com/personal/renjie_cui_business_uzh_ch/Documents/PeerGrading/Input/form_exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="318" documentId="8_{9C3C9BE7-B8B4-430B-A3DC-C1A29F196D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3EAD73C-6D11-41A0-9508-F46B9360AE44}"/>
+  <xr:revisionPtr revIDLastSave="333" documentId="8_{9C3C9BE7-B8B4-430B-A3DC-C1A29F196D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CBD8D65-4695-4C34-92BB-16C2C2188FF8}"/>
   <bookViews>
     <workbookView xWindow="17280" yWindow="-16200" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7518" uniqueCount="1423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7713" uniqueCount="1462">
   <si>
     <t>Responseid</t>
   </si>
@@ -4305,6 +4305,123 @@
   </si>
   <si>
     <t>2026-03-04T19:28:41.7544099Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:32:23.2161673Z</t>
+  </si>
+  <si>
+    <t>The information was well prepared and clearly presented.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:32:23.2162078Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:34:10.7835417Z</t>
+  </si>
+  <si>
+    <t>The speaker showed good confidence while presenting.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:34:10.7835848Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:35:18.4540848Z</t>
+  </si>
+  <si>
+    <t>Good balance between visuals and spoken explanation.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:35:18.4541380Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:36:42.3827453Z</t>
+  </si>
+  <si>
+    <t>The presentation was interesting and engaging.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:36:42.3828101Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:34.3910725Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:34.3911378Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:42.6974093Z</t>
+  </si>
+  <si>
+    <t>The presentation showed good preparation and effort.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:37:42.6974503Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:38:55.0830185Z</t>
+  </si>
+  <si>
+    <t>The speaker communicated the ideas clearly and effectively.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:38:55.0830703Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:39:43.5485937Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:39:43.5486326Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:40:29.1895567Z</t>
+  </si>
+  <si>
+    <t>The examples helped to understand the topic better.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:40:29.1896101Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:12.7058905Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:12.7059302Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:43.6373925Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:43.6374339Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:49.2567103Z</t>
+  </si>
+  <si>
+    <t>Very technical presentation but the key points were explained clearly and effectively.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:41:49.2567497Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:11.3387463Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:11.3387876Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:40.9457496Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:40.9457885Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:48.3346651Z</t>
+  </si>
+  <si>
+    <t>Well delivered and easy to follow.</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:42:48.3347398Z</t>
   </si>
 </sst>
 </file>
@@ -4408,8 +4525,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="responses" displayName="responses" ref="A1:N617" totalsRowShown="0">
-  <autoFilter ref="A1:N617" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="responses" displayName="responses" ref="A1:N632" totalsRowShown="0">
+  <autoFilter ref="A1:N632" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Responseid" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="SubmittedAt"/>
@@ -4727,7 +4844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N617"/>
+  <dimension ref="A1:N632"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="14" width="20" bestFit="1" customWidth="1"/>
@@ -31706,7 +31823,7 @@
       </c>
     </row>
     <row r="614" spans="1:14">
-      <c r="A614" s="5">
+      <c r="A614">
         <v>618</v>
       </c>
       <c r="B614" s="1" t="s">
@@ -31750,7 +31867,7 @@
       </c>
     </row>
     <row r="615" spans="1:14">
-      <c r="A615" s="5">
+      <c r="A615">
         <v>619</v>
       </c>
       <c r="B615" s="1" t="s">
@@ -31794,7 +31911,7 @@
       </c>
     </row>
     <row r="616" spans="1:14">
-      <c r="A616" s="5">
+      <c r="A616">
         <v>620</v>
       </c>
       <c r="B616" s="1" t="s">
@@ -31838,7 +31955,7 @@
       </c>
     </row>
     <row r="617" spans="1:14">
-      <c r="A617" s="5">
+      <c r="A617">
         <v>621</v>
       </c>
       <c r="B617" s="1" t="s">
@@ -31879,6 +31996,666 @@
       </c>
       <c r="N617" s="4" t="s">
         <v>1422</v>
+      </c>
+    </row>
+    <row r="618" spans="1:14">
+      <c r="A618" s="5">
+        <v>622</v>
+      </c>
+      <c r="B618" s="1" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C618" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D618" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E618" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G618" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H618" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J618" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L618" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M618" s="3" t="s">
+        <v>1424</v>
+      </c>
+      <c r="N618" s="4" t="s">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="619" spans="1:14">
+      <c r="A619" s="5">
+        <v>623</v>
+      </c>
+      <c r="B619" s="1" t="s">
+        <v>1426</v>
+      </c>
+      <c r="C619" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D619" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E619" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G619" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H619" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K619" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L619" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M619" s="3" t="s">
+        <v>1427</v>
+      </c>
+      <c r="N619" s="4" t="s">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="620" spans="1:14">
+      <c r="A620" s="5">
+        <v>624</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C620" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D620" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E620" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J620" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K620" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L620" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M620" s="3" t="s">
+        <v>1430</v>
+      </c>
+      <c r="N620" s="4" t="s">
+        <v>1431</v>
+      </c>
+    </row>
+    <row r="621" spans="1:14">
+      <c r="A621" s="5">
+        <v>625</v>
+      </c>
+      <c r="B621" s="1" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C621" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D621" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E621" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="F621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G621" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J621" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K621" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L621" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M621" s="3" t="s">
+        <v>1433</v>
+      </c>
+      <c r="N621" s="4" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="622" spans="1:14">
+      <c r="A622" s="5">
+        <v>626</v>
+      </c>
+      <c r="B622" s="1" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C622" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D622" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E622" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L622" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M622" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N622" s="4" t="s">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="623" spans="1:14">
+      <c r="A623" s="5">
+        <v>627</v>
+      </c>
+      <c r="B623" s="1" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C623" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D623" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E623" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="F623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J623" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L623" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M623" s="3" t="s">
+        <v>1438</v>
+      </c>
+      <c r="N623" s="4" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="624" spans="1:14">
+      <c r="A624" s="5">
+        <v>628</v>
+      </c>
+      <c r="B624" s="1" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C624" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D624" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E624" s="2" t="s">
+        <v>945</v>
+      </c>
+      <c r="F624" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L624" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M624" s="3" t="s">
+        <v>1441</v>
+      </c>
+      <c r="N624" s="4" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="625" spans="1:14">
+      <c r="A625" s="5">
+        <v>629</v>
+      </c>
+      <c r="B625" s="1" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C625" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D625" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E625" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L625" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M625" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N625" s="4" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="626" spans="1:14">
+      <c r="A626" s="5">
+        <v>630</v>
+      </c>
+      <c r="B626" s="1" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C626" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D626" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E626" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G626" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K626" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L626" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M626" s="3" t="s">
+        <v>1446</v>
+      </c>
+      <c r="N626" s="4" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="627" spans="1:14">
+      <c r="A627" s="5">
+        <v>631</v>
+      </c>
+      <c r="B627" s="1" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C627" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D627" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E627" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L627" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M627" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N627" s="4" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="628" spans="1:14">
+      <c r="A628" s="5">
+        <v>632</v>
+      </c>
+      <c r="B628" s="1" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C628" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D628" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E628" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="F628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L628" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M628" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N628" s="4" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="629" spans="1:14">
+      <c r="A629" s="5">
+        <v>633</v>
+      </c>
+      <c r="B629" s="1" t="s">
+        <v>1452</v>
+      </c>
+      <c r="C629" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D629" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E629" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="F629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H629" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I629" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L629" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M629" s="3" t="s">
+        <v>1453</v>
+      </c>
+      <c r="N629" s="4" t="s">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="630" spans="1:14">
+      <c r="A630" s="5">
+        <v>634</v>
+      </c>
+      <c r="B630" s="1" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C630" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D630" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E630" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="F630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L630" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M630" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N630" s="4" t="s">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="631" spans="1:14">
+      <c r="A631" s="5">
+        <v>635</v>
+      </c>
+      <c r="B631" s="1" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C631" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D631" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E631" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="F631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L631" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M631" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N631" s="4" t="s">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="632" spans="1:14">
+      <c r="A632" s="5">
+        <v>636</v>
+      </c>
+      <c r="B632" s="1" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C632" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D632" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E632" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="F632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L632" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="M632" s="3" t="s">
+        <v>1460</v>
+      </c>
+      <c r="N632" s="4" t="s">
+        <v>1461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync Forms export and update outputs (#9)
Co-authored-by: RenjieCui <71599592+RenjieCui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/PeerGrading/Input/form_exports/forms_responses.xlsx
+++ b/PeerGrading/Input/form_exports/forms_responses.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uzh-my.sharepoint.com/personal/renjie_cui_business_uzh_ch/Documents/PeerGrading/Input/form_exports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="333" documentId="8_{9C3C9BE7-B8B4-430B-A3DC-C1A29F196D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CBD8D65-4695-4C34-92BB-16C2C2188FF8}"/>
+  <xr:revisionPtr revIDLastSave="335" documentId="8_{9C3C9BE7-B8B4-430B-A3DC-C1A29F196D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{542380F8-6E33-415B-9FAD-32D7F529470C}"/>
   <bookViews>
     <workbookView xWindow="17280" yWindow="-16200" windowWidth="29010" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7713" uniqueCount="1462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7739" uniqueCount="1466">
   <si>
     <t>Responseid</t>
   </si>
@@ -4422,6 +4422,18 @@
   </si>
   <si>
     <t>2026-03-06T13:42:48.3347398Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:44:22.3693009Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:44:22.3693530Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:49:18.7307023Z</t>
+  </si>
+  <si>
+    <t>2026-03-06T13:49:18.7307458Z</t>
   </si>
 </sst>
 </file>
@@ -4525,8 +4537,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="responses" displayName="responses" ref="A1:N632" totalsRowShown="0">
-  <autoFilter ref="A1:N632" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="responses" displayName="responses" ref="A1:N634" totalsRowShown="0">
+  <autoFilter ref="A1:N634" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Responseid" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="SubmittedAt"/>
@@ -4844,7 +4856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N632"/>
+  <dimension ref="A1:N634"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="14" width="20" bestFit="1" customWidth="1"/>
@@ -32658,6 +32670,94 @@
         <v>1461</v>
       </c>
     </row>
+    <row r="633" spans="1:14">
+      <c r="A633" s="5">
+        <v>637</v>
+      </c>
+      <c r="B633" s="1" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C633" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D633" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E633" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="F633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L633" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M633" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N633" s="4" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="634" spans="1:14">
+      <c r="A634" s="5">
+        <v>638</v>
+      </c>
+      <c r="B634" s="1" t="s">
+        <v>1464</v>
+      </c>
+      <c r="C634" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D634" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E634" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="F634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L634" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M634" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="N634" s="4" t="s">
+        <v>1465</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>